<commit_message>
update evaluation for advisor
</commit_message>
<xml_diff>
--- a/LLM_judge_alignment/advisor_test_result/test_result_prompt_0.xlsx
+++ b/LLM_judge_alignment/advisor_test_result/test_result_prompt_0.xlsx
@@ -1064,11 +1064,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>acceptable</t>
         </is>
       </c>
       <c r="H6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1168,11 +1168,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1415,11 +1415,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>acceptable</t>
         </is>
       </c>
       <c r="H9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1766,11 +1766,11 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>acceptable</t>
+          <t>good</t>
         </is>
       </c>
       <c r="H12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1883,11 +1883,11 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>acceptable</t>
+          <t>good</t>
         </is>
       </c>
       <c r="H13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1909,11 +1909,11 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -2195,11 +2195,11 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="Z15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA15" t="inlineStr"/>
     </row>
@@ -2780,11 +2780,11 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>good</t>
+          <t>invalid</t>
         </is>
       </c>
       <c r="Z20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="inlineStr"/>
     </row>
@@ -3274,11 +3274,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -3313,11 +3313,11 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="N25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -3521,11 +3521,11 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="H27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -3599,11 +3599,11 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>acceptable</t>
+          <t>good</t>
         </is>
       </c>
       <c r="Z27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA27" t="inlineStr"/>
     </row>
@@ -3859,11 +3859,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>invalid</t>
+          <t>good</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -3872,11 +3872,11 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>acceptable</t>
+          <t>good</t>
         </is>
       </c>
       <c r="H30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>acceptable</t>
+          <t>invalid</t>
         </is>
       </c>
       <c r="Q31" t="b">

</xml_diff>